<commit_message>
Avaliações AV Wyden UniRuy 2025.2 - 02122025 ...
</commit_message>
<xml_diff>
--- a/03 Assessments/Turma Python Paradigmas - 3001 Wyden UniRuy 2025_2.xlsx
+++ b/03 Assessments/Turma Python Paradigmas - 3001 Wyden UniRuy 2025_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heleno\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7254DAA6-EDB6-47F0-B424-5B2946274A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E300A2ED-44A6-4BA2-8864-8E85FDE9DCA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{DD6ED3E7-57DF-4A52-9E4C-63B0F7661B3D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="50">
   <si>
     <t>-</t>
   </si>
@@ -47,9 +47,6 @@
     <t>AV</t>
   </si>
   <si>
-    <t>AVS</t>
-  </si>
-  <si>
     <t>SIM1</t>
   </si>
   <si>
@@ -86,18 +83,12 @@
     <t>202505116773 - DAVI DOS SANTOS DE OLIVEIRA</t>
   </si>
   <si>
-    <t>202502388251 - DEUSINETE DE JESUS DUTRA</t>
-  </si>
-  <si>
     <t>202503582734 - ERIC ASSIS DOS SANTOS SILVA</t>
   </si>
   <si>
     <t>202502843798 - ERICK ROCHA LUCIANO NASCIMENTO</t>
   </si>
   <si>
-    <t>202403650223 - ERIK MATOS</t>
-  </si>
-  <si>
     <t>202402969821 - FELIPE DANTAS RIBEIRO DOS SANTOS</t>
   </si>
   <si>
@@ -135,9 +126,6 @@
   </si>
   <si>
     <t>202503547106 - RENATA DA CONCEICAO MACHADO</t>
-  </si>
-  <si>
-    <t>202504001174 - RENATO MACHADO DOS SANTOS JUNIOR</t>
   </si>
   <si>
     <t>202503356751 - RODRIGO SANTOS ARAÚJO</t>
@@ -256,6 +244,18 @@
       </rPr>
       <t>; https://github.com/ThalesAlexandreSoares/task-manager</t>
     </r>
+  </si>
+  <si>
+    <t>TRAB</t>
+  </si>
+  <si>
+    <t>202403650223 - ERIK MATOS AVS = 2,1</t>
+  </si>
+  <si>
+    <t>202504001174 - RENATO MACHADO DOS SANTOS JUNIOR AVS = 2,1</t>
+  </si>
+  <si>
+    <t>202502388251 - DEUSINETE DE JESUS DUTRA  AVS = 4,9</t>
   </si>
 </sst>
 </file>
@@ -900,7 +900,8 @@
     <col min="2" max="2" width="11.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24.85546875" style="2" bestFit="1" customWidth="1"/>
@@ -909,13 +910,13 @@
   <sheetData>
     <row r="1" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D1" s="14" t="s">
         <v>3</v>
@@ -924,21 +925,21 @@
         <v>4</v>
       </c>
       <c r="F1" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="15" t="s">
-        <v>6</v>
-      </c>
       <c r="I1" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="17">
         <v>3.5</v>
@@ -953,23 +954,24 @@
       <c r="E2" s="17">
         <v>0.6</v>
       </c>
-      <c r="F2" s="17" t="s">
-        <v>1</v>
+      <c r="F2" s="17">
+        <f>G2</f>
+        <v>2.8</v>
       </c>
       <c r="G2" s="17">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H2" s="18">
         <f>C2+G2</f>
-        <v>2</v>
+        <v>4.8</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="19" t="s">
         <v>1</v>
@@ -993,12 +995,12 @@
         <v>0</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="7">
         <v>5.6</v>
@@ -1024,12 +1026,12 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="B5" s="7">
         <v>4.2</v>
@@ -1055,12 +1057,12 @@
         <v>2.4</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B6" s="7">
         <v>6.3</v>
@@ -1086,12 +1088,12 @@
         <v>9.6</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>1</v>
@@ -1115,12 +1117,12 @@
         <v>0</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="B8" s="7">
         <v>3.5</v>
@@ -1146,12 +1148,12 @@
         <v>2</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B9" s="7">
         <v>6.3</v>
@@ -1177,12 +1179,12 @@
         <v>9.6</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>1</v>
@@ -1206,12 +1208,12 @@
         <v>0</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>1</v>
@@ -1235,12 +1237,12 @@
         <v>0</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>1</v>
@@ -1264,12 +1266,12 @@
         <v>0</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B13" s="7">
         <v>5.6</v>
@@ -1295,12 +1297,12 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B14" s="7">
         <v>6.3</v>
@@ -1326,12 +1328,12 @@
         <v>9.6</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B15" s="7">
         <v>5.6</v>
@@ -1357,12 +1359,12 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B16" s="7">
         <v>5.6</v>
@@ -1388,12 +1390,12 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B17" s="7">
         <v>4.9000000000000004</v>
@@ -1419,12 +1421,12 @@
         <v>8.8000000000000007</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B18" s="7">
         <v>5.6</v>
@@ -1450,12 +1452,12 @@
         <v>8.6999999999999993</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B19" s="7">
         <v>4.2</v>
@@ -1481,12 +1483,12 @@
         <v>8.4</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="16" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B20" s="19" t="s">
         <v>1</v>
@@ -1510,12 +1512,12 @@
         <v>0</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B21" s="7">
         <v>4.9000000000000004</v>
@@ -1541,12 +1543,12 @@
         <v>8.8000000000000007</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="B22" s="7">
         <v>4.9000000000000004</v>
@@ -1572,12 +1574,12 @@
         <v>2.8000000000000003</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B23" s="7">
         <v>4.9000000000000004</v>
@@ -1603,12 +1605,12 @@
         <v>8.8000000000000007</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B24" s="8">
         <v>6.3</v>
@@ -1634,12 +1636,12 @@
         <v>9.6</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -1647,15 +1649,15 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>